<commit_message>
Read DWG directly, consultant layer profiles, AashirTools-style ribbon
- ACadSharp 3.6.35 (same pinned version as AashirTools) reads DWG
  in-process; ODA/AutoCAD only as fallback. Markup DWG also written
  with ACadSharp. Streams are opened explicitly so no file stays locked.
- Layer classification: consultant profile (review grid, saved once in
  %APPDATA%\RevitCadQC\CadProfiles) > CadLayerDictionary.txt (first
  match wins) > built-in rules; unknown layers skipped, never guessed
- Layer review shown automatically for a new consultant; Layer Mapping,
  Layer Dictionary and Version buttons; 96px vector icons
- Team package carries the dictionary and consultant profiles
- .addin uses AddInId; tests for DWG input, dictionary and profiles

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QgTPzTFL3ce6jdDoFGdnL
</commit_message>
<xml_diff>
--- a/RevitCadQC/docs/sample-output/QC_Issues.xlsx
+++ b/RevitCadQC/docs/sample-output/QC_Issues.xlsx
@@ -128,7 +128,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/tmp/cadqc_test_f36f12f11ff549d595f4afdc0e473ee6</t>
+          <t xml:space="preserve">/tmp/cadqc_test_30b4df8eb6f1447fa9645dbda136e348</t>
         </is>
       </c>
     </row>
@@ -140,7 +140,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-26 03:23</t>
+          <t xml:space="preserve">2026-09-26 05:08</t>
         </is>
       </c>
     </row>
@@ -151,7 +151,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7"/>

</xml_diff>

<commit_message>
Restructure like AashirTools, add update system, central config, CAD links
- One project at the root (Commands/, Core/, UI/), one RevitCadQC.dll,
  dotnet build -c R2022..R2026 -> bin\R20xx; tests and CLI compile Core
- Check for Update + start-up check from the team package folder
  (version.txt, FORCE silent update, NEWPATH redirect, .old DLL swap)
- CadQcConfig.txt central office rules (defaults and !enforced keys),
  read live from the team package
- CAD linked in the model is checked at its link placement (exact
  alignment candidate, auto-alignment still competes)
- Scripts rewritten for the new layout; team package writes version.txt
  from Core\ToolVersion.cs and deploys to TEAM_DEPLOY_PATHS.txt
- net48 builds reference System.IO.Compression (Excel export)
- 41 tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QgTPzTFL3ce6jdDoFGdnL
</commit_message>
<xml_diff>
--- a/RevitCadQC/docs/sample-output/QC_Issues.xlsx
+++ b/RevitCadQC/docs/sample-output/QC_Issues.xlsx
@@ -128,7 +128,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">/tmp/cadqc_test_30b4df8eb6f1447fa9645dbda136e348</t>
+          <t xml:space="preserve">/tmp/cadqc_test_87e50d611c58425f99107f1094424321</t>
         </is>
       </c>
     </row>
@@ -140,7 +140,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-26 05:08</t>
+          <t xml:space="preserve">2026-09-26 05:23</t>
         </is>
       </c>
     </row>
@@ -151,7 +151,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7"/>

</xml_diff>